<commit_message>
S7: fix integration findings in S2/S3/S4/S5 and use S4 yaw for exclusion zones
- S3: remove stray empty "tests/test data"; add src/open_vocab/README.md
- S2: update paths to S3's moved contract/pipeline files
- S4: export node yaw (box rotation about z); regenerate frame_000 scene graph
- S5: closest-object queries skip virtual nodes (desk plane) unless named; add test
- S6 placeholder: exclusion zones are the yaw-rotated footprint (square fallback without yaw)
- S7: live S3 uses desk.json prompts; eval set +1 query; refreshed experiment matrix and docs

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WtjFQe5gesQc7m5LhgwAQ8
</commit_message>
<xml_diff>
--- a/outputs/evaluation/experiment_matrix.xlsx
+++ b/outputs/evaluation/experiment_matrix.xlsx
@@ -479,7 +479,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>839.61</v>
+        <v>757.47</v>
       </c>
     </row>
     <row r="6">
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1.191</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="7">
@@ -499,7 +499,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>14.58</v>
+        <v>14.44</v>
       </c>
     </row>
     <row r="8">
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4.96</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="9">
@@ -519,7 +519,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>819.53</v>
+        <v>737.86</v>
       </c>
     </row>
     <row r="10">
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="11">
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.49</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="12">
@@ -569,7 +569,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15">
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17">
@@ -643,7 +643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -797,10 +797,10 @@
         <v>0</v>
       </c>
       <c r="N2" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="O2" t="n">
         <v>0.1</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0.07000000000000001</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
@@ -859,10 +859,10 @@
         <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="O3" t="n">
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
@@ -918,10 +918,10 @@
         <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.11</v>
       </c>
       <c r="O4" t="n">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
@@ -980,7 +980,7 @@
         <v>0.1</v>
       </c>
       <c r="O5" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
@@ -1039,10 +1039,10 @@
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="O6" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
@@ -1053,17 +1053,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Where is the multimeter?</t>
+          <t>What is closest to the book?</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>multimeter</t>
+          <t>mug</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>multimeter_01</t>
+          <t>mug_01</t>
         </is>
       </c>
       <c r="D7" t="b">
@@ -1074,14 +1074,14 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>multimeter</t>
+          <t>desk</t>
         </is>
       </c>
       <c r="G7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I7" t="b">
         <v>1</v>
@@ -1101,31 +1101,31 @@
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="O7" t="n">
-        <v>0.06</v>
+        <v>0.09</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>The multimeter is multimeter_01 at x=0.47, y=0.10, z=0.03 m, on desk_01.</t>
+          <t>The closest object to the book is mug_01, verified at 0.30 meters.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Find the book that is not near the mug</t>
+          <t>Where is the multimeter?</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>book</t>
+          <t>multimeter</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>book_01</t>
+          <t>multimeter_01</t>
         </is>
       </c>
       <c r="D8" t="b">
@@ -1136,14 +1136,14 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>laptop</t>
+          <t>multimeter</t>
         </is>
       </c>
       <c r="G8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I8" t="b">
         <v>1</v>
@@ -1163,32 +1163,42 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="O8" t="n">
         <v>0.09</v>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>book_01 is a book that is NOT near the mug.</t>
+          <t>The multimeter is multimeter_01 at x=0.47, y=0.10, z=0.03 m, on desk_01.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Find a cup that is not near the laptop</t>
+          <t>Find the book that is not near the mug</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>book</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>book_01</t>
         </is>
       </c>
       <c r="D9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" t="b">
         <v>1</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>mug</t>
+          <t>laptop</t>
         </is>
       </c>
       <c r="G9" t="b">
@@ -1198,35 +1208,38 @@
         <v>1</v>
       </c>
       <c r="I9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>S5 could not verify a target; no goal sent to the virtual agent</t>
+          <t>path is clear</t>
         </is>
       </c>
       <c r="L9" t="b">
+        <v>1</v>
+      </c>
+      <c r="M9" t="n">
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>0.11</v>
+        <v>0.18</v>
       </c>
       <c r="O9" t="n">
-        <v>0.01</v>
+        <v>0.13</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Cannot determine: no object satisfies the constraint.</t>
+          <t>book_01 is a book that is NOT near the mug.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Which chair is closest to the laptop?</t>
+          <t>Find a cup that is not near the laptop</t>
         </is>
       </c>
       <c r="D10" t="b">
@@ -1237,7 +1250,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>chair</t>
+          <t>mug</t>
         </is>
       </c>
       <c r="G10" t="b">
@@ -1261,61 +1274,110 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
       <c r="O10" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Cannot determine: no matching objects in the scene graph.</t>
+          <t>Cannot determine: no object satisfies the constraint.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Which chair is closest to the laptop?</t>
+        </is>
+      </c>
+      <c r="D11" t="b">
+        <v>0</v>
+      </c>
+      <c r="E11" t="b">
+        <v>1</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>chair</t>
+        </is>
+      </c>
+      <c r="G11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I11" t="b">
+        <v>0</v>
+      </c>
+      <c r="J11" t="b">
+        <v>0</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>S5 could not verify a target; no goal sent to the virtual agent</t>
+        </is>
+      </c>
+      <c r="L11" t="b">
+        <v>0</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Cannot determine: no matching objects in the scene graph.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>Where is the red stapler?</t>
         </is>
       </c>
-      <c r="D11" t="b">
-        <v>0</v>
-      </c>
-      <c r="E11" t="b">
-        <v>1</v>
-      </c>
-      <c r="F11" t="inlineStr">
+      <c r="D12" t="b">
+        <v>0</v>
+      </c>
+      <c r="E12" t="b">
+        <v>1</v>
+      </c>
+      <c r="F12" t="inlineStr">
         <is>
           <t>stapler</t>
         </is>
       </c>
-      <c r="G11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I11" t="b">
-        <v>0</v>
-      </c>
-      <c r="J11" t="b">
-        <v>0</v>
-      </c>
-      <c r="K11" t="inlineStr">
+      <c r="G12" t="b">
+        <v>1</v>
+      </c>
+      <c r="H12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I12" t="b">
+        <v>0</v>
+      </c>
+      <c r="J12" t="b">
+        <v>0</v>
+      </c>
+      <c r="K12" t="inlineStr">
         <is>
           <t>S5 could not verify a target; no goal sent to the virtual agent</t>
         </is>
       </c>
-      <c r="L11" t="b">
-        <v>0</v>
-      </c>
-      <c r="N11" t="n">
+      <c r="L12" t="b">
+        <v>0</v>
+      </c>
+      <c r="N12" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="O11" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="P11" t="inlineStr">
+      <c r="O12" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="P12" t="inlineStr">
         <is>
           <t>Cannot determine: 'stapler' is not in the scene graph.</t>
         </is>
@@ -1412,22 +1474,22 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>19.2</v>
+        <v>18.84</v>
       </c>
       <c r="E2" t="n">
-        <v>4.89</v>
+        <v>4.87</v>
       </c>
       <c r="F2" t="n">
-        <v>1337.49</v>
+        <v>1212.17</v>
       </c>
       <c r="G2" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="H2" t="n">
-        <v>1.18</v>
+        <v>1.05</v>
       </c>
       <c r="I2" t="n">
-        <v>1362.82</v>
+        <v>1236.99</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -1448,22 +1510,22 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>13.03</v>
+        <v>12.62</v>
       </c>
       <c r="E3" t="n">
-        <v>4.39</v>
+        <v>4.27</v>
       </c>
       <c r="F3" t="n">
-        <v>684.91</v>
+        <v>666.46</v>
       </c>
       <c r="G3" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>0.39</v>
+        <v>0.65</v>
       </c>
       <c r="I3" t="n">
-        <v>702.79</v>
+        <v>684.0599999999999</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -1484,22 +1546,22 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>14.46</v>
+        <v>13.13</v>
       </c>
       <c r="E4" t="n">
-        <v>5.63</v>
+        <v>5.02</v>
       </c>
       <c r="F4" t="n">
-        <v>722.72</v>
+        <v>724.64</v>
       </c>
       <c r="G4" t="n">
-        <v>0.09</v>
+        <v>0.03</v>
       </c>
       <c r="H4" t="n">
-        <v>0.4</v>
+        <v>0.49</v>
       </c>
       <c r="I4" t="n">
-        <v>743.29</v>
+        <v>743.3099999999999</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -1520,22 +1582,22 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>14.41</v>
+        <v>15.98</v>
       </c>
       <c r="E5" t="n">
-        <v>6.62</v>
+        <v>6.13</v>
       </c>
       <c r="F5" t="n">
-        <v>970.65</v>
+        <v>671.3099999999999</v>
       </c>
       <c r="G5" t="n">
         <v>0.04</v>
       </c>
       <c r="H5" t="n">
-        <v>0.4</v>
+        <v>0.39</v>
       </c>
       <c r="I5" t="n">
-        <v>992.12</v>
+        <v>693.86</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -1556,22 +1618,22 @@
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>13.12</v>
+        <v>13.22</v>
       </c>
       <c r="E6" t="n">
-        <v>3.77</v>
+        <v>3.49</v>
       </c>
       <c r="F6" t="n">
-        <v>638.01</v>
+        <v>615.05</v>
       </c>
       <c r="G6" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="H6" t="n">
-        <v>0.32</v>
+        <v>0.38</v>
       </c>
       <c r="I6" t="n">
-        <v>655.26</v>
+        <v>632.17</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -1592,22 +1654,22 @@
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>15.85</v>
+        <v>12.68</v>
       </c>
       <c r="E7" t="n">
-        <v>4.76</v>
+        <v>3.44</v>
       </c>
       <c r="F7" t="n">
-        <v>776.49</v>
+        <v>581.8099999999999</v>
       </c>
       <c r="G7" t="n">
         <v>0.04</v>
       </c>
       <c r="H7" t="n">
-        <v>0.42</v>
+        <v>0.31</v>
       </c>
       <c r="I7" t="n">
-        <v>797.5599999999999</v>
+        <v>598.28</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -1628,22 +1690,22 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>13.24</v>
+        <v>13.2</v>
       </c>
       <c r="E8" t="n">
-        <v>4.6</v>
+        <v>4.91</v>
       </c>
       <c r="F8" t="n">
-        <v>698.9299999999999</v>
+        <v>753.15</v>
       </c>
       <c r="G8" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="H8" t="n">
-        <v>0.48</v>
+        <v>0.49</v>
       </c>
       <c r="I8" t="n">
-        <v>717.29</v>
+        <v>771.79</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -1664,22 +1726,22 @@
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>13.3</v>
+        <v>15.86</v>
       </c>
       <c r="E9" t="n">
-        <v>5.02</v>
+        <v>4.68</v>
       </c>
       <c r="F9" t="n">
-        <v>727.02</v>
+        <v>678.29</v>
       </c>
       <c r="G9" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="H9" t="n">
-        <v>0.36</v>
+        <v>0.4</v>
       </c>
       <c r="I9" t="n">
-        <v>745.78</v>
+        <v>699.27</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>

</xml_diff>